<commit_message>
Updated SauceDemo login test cases
</commit_message>
<xml_diff>
--- a/SauceDemo_Login-TEST_Cases.xlsx
+++ b/SauceDemo_Login-TEST_Cases.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="80">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -41,13 +41,252 @@
   </si>
   <si>
     <t>Priority</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_001</t>
+  </si>
+  <si>
+    <t>Login</t>
+  </si>
+  <si>
+    <t>Verify login with valid credentials</t>
+  </si>
+  <si>
+    <t>User is on SauceDemo login page</t>
+  </si>
+  <si>
+    <t>1. Enter username
+2. Enter password
+3. Click Login</t>
+  </si>
+  <si>
+    <t>username: standard_user
+password: secret_sauce</t>
+  </si>
+  <si>
+    <t>User should successfully login and navigate to Products page</t>
+  </si>
+  <si>
+    <t>User successfully logged in and was redirected to the Products page (https://www.saucedemo.com/inventory.html). All 6 products were displayed correctly with images, descriptions, prices, and Add to Cart buttons. Cart icon displayed "0" initially.</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_002</t>
+  </si>
+  <si>
+    <t>Verify login with invalid credentials</t>
+  </si>
+  <si>
+    <t>1. Enter invalid username
+2. Enter invalid password
+3. Click 'Login' button</t>
+  </si>
+  <si>
+    <t>username: invalid_user
+password: wrong_password</t>
+  </si>
+  <si>
+    <t>An error messaage should be displayed:"Username and password do not match any user in this service.". User should remain on the login page</t>
+  </si>
+  <si>
+    <t>Error message displayed: "Epic sadface: Username and password do not match any user in this service" . User remained on the login page. URL did not change (https://www.saucedemo.com/).</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_003</t>
+  </si>
+  <si>
+    <t>Verify login with empty credentials</t>
+  </si>
+  <si>
+    <t>1. Leave username and password fields empty
+2. Click 'Login' button</t>
+  </si>
+  <si>
+    <t>username: 
+password:</t>
+  </si>
+  <si>
+    <t>An error message should be displayed: "Username is required." User should remain on the login page.</t>
+  </si>
+  <si>
+    <t>Error message displayed: "Epic sadface: Username is required" . User remained on the login page. URL did not change. Both fields remained empty and no redirection occurred.</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_004</t>
+  </si>
+  <si>
+    <t>Verify login with locked-out user</t>
+  </si>
+  <si>
+    <t>1. Enter locked-out username
+2. Enter valid password
+3. Click 'Login' button</t>
+  </si>
+  <si>
+    <t>username: locked_out_user
+password: secret_sauce</t>
+  </si>
+  <si>
+    <t>An error message should be displayed: "Sorry, this user has been locked out." User should remain on the login page.</t>
+  </si>
+  <si>
+    <t>Error message displayed: "Epic sadface: Sorry, this user has been locked out" . User remained on the login page. URL did not change. Login was prevented as expected.</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_005</t>
+  </si>
+  <si>
+    <t>Verify login with valid username and empty password</t>
+  </si>
+  <si>
+    <t>1. Enter valid username
+2. Leave password field empty
+3. Click 'Login' button</t>
+  </si>
+  <si>
+    <t>username: standard_user
+password:</t>
+  </si>
+  <si>
+    <t>Error message should be displayed: "Epic sadface: Password is required" . User should remain on login page.</t>
+  </si>
+  <si>
+    <t>Error message displayed: "Epic sadface: Password is required" . User remained on the login page. URL did not change. Password field remained empty and no redirection occurred.</t>
+  </si>
+  <si>
+    <t>pass</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_006</t>
+  </si>
+  <si>
+    <t>Verify login with valid username and invalid password</t>
+  </si>
+  <si>
+    <t>1. Enter valid username
+2. Enter invalid password
+3. Click 'Login' button</t>
+  </si>
+  <si>
+    <t>username: standard_user
+password: wrong_passwprd</t>
+  </si>
+  <si>
+    <t>Error message should be displayed: "Epic sadface: Username and password do not match any user in this service" . User should remain on login page.</t>
+  </si>
+  <si>
+    <t>Error message displayed: "Epic sadface: Username and password do not match any user in this service" . User remained on the login page. URL did not change. Login was prevented as expected.</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_007</t>
+  </si>
+  <si>
+    <t>Verify login with problem user</t>
+  </si>
+  <si>
+    <t>1. Enter problem user username
+2. Enter valid password
+3. Click 'Login' button</t>
+  </si>
+  <si>
+    <t>username: problem_user
+password: secret_sauce</t>
+  </si>
+  <si>
+    <t>User should login successfully BUT may experience visual glitches or broken images on the products page (known issue with this user). Login should still be successful.</t>
+  </si>
+  <si>
+    <t>User logged in successfully and navigated to Products page. However, product images were broken/replaced with placeholder icons on the inventory page. Product names and prices were displayed correctly.</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_008</t>
+  </si>
+  <si>
+    <t>Verify login with performance glitch user</t>
+  </si>
+  <si>
+    <t>1. Enter performance glitch user username
+2. Enter valid password
+3. Click 'Login' button</t>
+  </si>
+  <si>
+    <t>username: performance_glitch_user
+password: secret_sauce</t>
+  </si>
+  <si>
+    <t>User should login successfully but may experience significant delay (approx. 5+ seconds) before redirecting to products page. Login should eventually succeed.</t>
+  </si>
+  <si>
+    <t>Login took approximately 5-8 seconds to complete. User eventually navigated to Products page successfully. All images and functionality loaded correctly after the delay.</t>
+  </si>
+  <si>
+    <t>Pass(login successful with performance delay)</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_009</t>
+  </si>
+  <si>
+    <t>Verify login with error user</t>
+  </si>
+  <si>
+    <t>1. Enter error user username
+2. Enter valid password
+3. Click 'Login' button</t>
+  </si>
+  <si>
+    <t>username: error_user
+password: secret_sauce</t>
+  </si>
+  <si>
+    <t>User should login successfully BUT may encounter various errors or broken functionality on the products page (known issue). Login itself should be successful.</t>
+  </si>
+  <si>
+    <t>User logged in successfully and navigated to Products page. Add to Cart button for Sauce Labs Backpack was missing. Some images were broken. Multiple elements had incorrect styling or were unresponsive.</t>
+  </si>
+  <si>
+    <t>Pass (Login successful, but multiple UI/functional defects present)</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_010</t>
+  </si>
+  <si>
+    <t>Verify login with visual user</t>
+  </si>
+  <si>
+    <t>1. Enter visual user username
+2. Enter valid password
+3. Click 'Login' button</t>
+  </si>
+  <si>
+    <t>username: visual_user
+password: secret_sauce</t>
+  </si>
+  <si>
+    <t>User should login successfully but the UI may appear differently (e.g., missing images, different button colors - known visual testing user). Login should be successful.</t>
+  </si>
+  <si>
+    <t>User logged in successfully and navigated to Products page. All product images had different sizes/shapes than standard_user. Add to Cart buttons were styled differently (different colors and margins). The overall layout appeared distorted.</t>
+  </si>
+  <si>
+    <t>Pass (Login successful, but visual differences present)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -55,17 +294,33 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11.0"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
+      <sz val="11.0"/>
+      <color rgb="FF0F1115"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="lightGray"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -74,11 +329,17 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -297,6 +558,17 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="13.25"/>
+    <col customWidth="1" min="2" max="2" width="27.75"/>
+    <col customWidth="1" min="3" max="3" width="44.63"/>
+    <col customWidth="1" min="4" max="4" width="30.0"/>
+    <col customWidth="1" min="5" max="5" width="35.25"/>
+    <col customWidth="1" min="6" max="6" width="28.0"/>
+    <col customWidth="1" min="7" max="7" width="125.25"/>
+    <col customWidth="1" min="8" max="8" width="203.0"/>
+    <col customWidth="1" min="9" max="9" width="48.75"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
@@ -330,6 +602,329 @@
         <v>9</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3"/>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>